<commit_message>
Consolidar nomes de orientadores: 111 → 83 únicos (28 variações unificadas)
</commit_message>
<xml_diff>
--- a/outputs/analise/corpus_tccs_analisado.xlsx
+++ b/outputs/analise/corpus_tccs_analisado.xlsx
@@ -953,7 +953,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor  José García Mendoza</t>
+          <t>Prof. Dr. Héctor José García  Mendoza</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Prof. Dr. Ricardo Carvalho dos Santos</t>
+          <t>Dr. Ricardo Carvalho dos Santos.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Prof. Dr. Ricardo Carvalho dos Santos</t>
+          <t>Dr. Ricardo Carvalho dos Santos.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1686,7 +1686,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Prof. Dr. Ricardo Carvalho dos Santos</t>
+          <t>Dr. Ricardo Carvalho dos Santos.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1976,7 +1976,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Prof. Dr. Ricardo Carvalho dos Santos</t>
+          <t>Dr. Ricardo Carvalho dos Santos.</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Danielle Trindade.</t>
+          <t>Danielle Trindade</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Profa. Dra. Eliaine de Morais Belford Gomes</t>
+          <t>Prof.a Dr.a Eliaine de Morais Belford Gomes</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -3138,7 +3138,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor José García  Mendoza</t>
+          <t>Prof. Dr. Héctor José García Mendoza</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -3432,7 +3432,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Profa. Dra. Cinara Franco Rechico Barberena</t>
+          <t>Prof.ª Dra. Cinara Franco Rechico Barberena</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -3873,7 +3873,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Prof. Dr. João Paulino da Silva Neto</t>
+          <t>Prof.o Dr. João Paulino da Silva Neto.</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -4020,7 +4020,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Prof. Dr. Maxim Repetto.</t>
+          <t>Prof Dr. Maxim Repetto.</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -4169,7 +4169,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Profa. Dra. Iana dos Santos Vasconcelos.</t>
+          <t>Dra. Iana dos Santos Vasconcelos</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -4465,7 +4465,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Prof. Dr. Maxim Repetto.</t>
+          <t>Prof Dr. Maxim Repetto.</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Professor Dr. Maxim Repetto Carreno</t>
+          <t>Prof. Dr. Maxim Repetto Carrreno</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -5206,7 +5206,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Prof. Dr. Sebastião Monteiro Oliveira2</t>
+          <t>Profº Msc. Dr. Sebastião Oliveira Monteiro</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -5643,7 +5643,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Edlauva Oliveira dos Santos.</t>
+          <t>Profª Dr. Edlauva Oliveira dos Santos</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -6368,7 +6368,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Prof. Dr. João Paulino da Silva Neto</t>
+          <t>Prof.o Dr. João Paulino da Silva Neto.</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -6513,7 +6513,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Prof. Dr. João Paulino da Silva Neto</t>
+          <t>Prof.o Dr. João Paulino da Silva Neto.</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -6948,7 +6948,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Pedro Augusto Hercks Menin</t>
+          <t>Prof. Dr. Pedro Augusto Hercks Menin</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -7381,7 +7381,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Profª Dr. Edlauva Oliveira dos Santos</t>
+          <t>Prof.a Dr.a Edlauva Oliveira dos Santos</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -7961,7 +7961,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Profa. Dra. Zoraide dos Anjos Gonçalves da Silva Vieira.</t>
+          <t>Profa. Dra. Zoraide  dos Anjos Gonçalves da Silva Vieira</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -8106,7 +8106,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Prof. Me. Celino Alexandre Raposo</t>
+          <t>Prof. Msc. Celino Alexandre Raposo</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -8396,7 +8396,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Dra. Zoraide dos Anjos Gonçalves Silva Vieira.</t>
+          <t>Profa. Dra. Zoraide dos Anjos Gonçalves da Silva Vieira.</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -9687,7 +9687,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Prof. Fábio Almeida de Carvalho</t>
+          <t>Prof.Dr. Fábio Almeida  de Carvalho</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -9832,7 +9832,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Profa Dra Ananda Machado</t>
+          <t>Profa Dra Ananda Machado.</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -10122,7 +10122,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Prof Dr. Jonildo Viana dos Santos.</t>
+          <t>Prof. Dr. Jonildo Viana dos Santos</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -10408,7 +10408,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Prof Dr. Maxim Repetto.</t>
+          <t>Prof. Maxim Repetto</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -10694,7 +10694,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Profa Dra. Fabíola Christian Almeida de Carvalho</t>
+          <t>Fabíola Christian Almeida de Carvalho</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -10980,7 +10980,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Prof. Dr. Jonildo Viana dos Santos.</t>
+          <t>Prof. Dr. Jonildo Viana  dos Santos.</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -11266,7 +11266,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Prof.ª Msc. Mariana Souza da Cunha</t>
+          <t>Prof.a Me. Mariana Souza da Cunha.</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Prof.a Dr.a Fabíola C. Almeida de Carvalho</t>
+          <t>Prof.Dr. Fábio Almeida  de Carvalho</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -11695,7 +11695,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Prof. Me. Mariana Souza da Cunha</t>
+          <t>Prof.ª Msc. Mariana Souza da Cunha</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -11838,7 +11838,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Prof. Dr. Ricardo Carvalho dos Santos</t>
+          <t>Dr. Ricardo Carvalho dos Santos.</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -11981,7 +11981,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Prof.a Me. Mariana Souza da Cunha.</t>
+          <t>Prof.a Mariana Souza da Cunha</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -12267,7 +12267,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Dr. Ricardo Carvalho dos Santos.</t>
+          <t>Ricardo Carvalho dos Santos</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -12410,7 +12410,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Prof. Dr. Rafael Branquinho Abdala Norberto.</t>
+          <t>Prof. Dr. Rafael Branquinho Abdala Norberto</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -12553,7 +12553,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Prof. M.e Jefferson Tiago de Souza Mendes da Silva</t>
+          <t>Orientador: Prof. Dr. Jefferson Tiago de Souza Mendes da Silva</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -12839,7 +12839,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Profa. Dra. Jéssica de Almeida.</t>
+          <t>Prof. Dra. Jéssica de Almeida</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -13554,7 +13554,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Prof. Dr. Rafael Branquinho Abdala Norberto.</t>
+          <t>Prof. Dr. Rafael Branquinho Abdala Norberto</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -13697,7 +13697,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Prof. Dra. Jéssica de Almeida</t>
+          <t>Prof.a Dra Jéssica de Almeida</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -13840,7 +13840,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Prof. M.a. Jéssica de Almeida</t>
+          <t>Prof. Dra. Jéssica de Almeida</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -13983,7 +13983,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Prof. Dra. Jessica de Almeida</t>
+          <t>Profa. Dra. Jéssica de Almeida.</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -14412,7 +14412,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Prof. Dr. Rafael Branquinho Abdala Norberto.</t>
+          <t>Prof. Dr. Rafael Branquinho Abdala Norberto</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -14555,7 +14555,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Jefferson Tiago de Souza Mendes da Silva</t>
+          <t>Prof. M.e Jefferson Tiago de Souza Mendes da Silva</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -16567,7 +16567,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>Profº Msc. Dr. Sebastião Oliveira Monteiro</t>
+          <t>Prof. Dr. Sebastião Monteiro Oliveira</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
@@ -16710,7 +16710,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Prof.ª Dr.ª Maria Edith Romano Siems Marcondes</t>
+          <t>Prof.ª Dr.ª Maria Edith Romano Siems-Marcondes</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -17572,7 +17572,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>Prof.ª Drº. Michael Lopes da Silva Rolim</t>
+          <t>Prof. Dr. Michael Lopes da Silva Rolim</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -17717,7 +17717,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>Prof. Dr.  Héctor José García Mendoza.</t>
+          <t>Prof. Dr. Héctor José García Mendoza.</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -17862,7 +17862,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor José  García Mendoza</t>
+          <t>Prof. Dr.  Héctor José García Mendoza.</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -18007,7 +18007,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor José García  Mendoza</t>
+          <t>Prof. Dr. Héctor José García Mendoza</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -18152,7 +18152,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor José García Mendoza.</t>
+          <t>Prof. Dr. Héctor  José García Mendoza</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -18297,7 +18297,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor José García Mendoza.</t>
+          <t>Prof. Dr. Héctor  José García Mendoza</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -18442,7 +18442,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor José García Mendoza.</t>
+          <t>Prof. Dr. Héctor  José García Mendoza</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -18732,7 +18732,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor José García Mendoza.</t>
+          <t>Prof. Dr. Héctor  José García Mendoza</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -18877,7 +18877,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor José García  Mendoza</t>
+          <t>Prof. Dr. Héctor José García Mendoza</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -19022,7 +19022,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor José  García Mendoza</t>
+          <t>Prof. Dr.  Héctor José García Mendoza.</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -19192,10 +19192,8 @@
           <t>1º semestre</t>
         </is>
       </c>
-      <c r="L130" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
+      <c r="L130" t="n">
+        <v>24</v>
       </c>
       <c r="M130" t="inlineStr">
         <is>
@@ -19232,13 +19230,17 @@
           <t>https://drive.google.com/file/d/1VUiHFakIErwS7hOIOikZDUdIEaf3bNYO/view?usp=sharing</t>
         </is>
       </c>
-      <c r="T130" t="inlineStr"/>
+      <c r="T130" t="n">
+        <v/>
+      </c>
       <c r="U130" t="inlineStr">
         <is>
           <t>Elcio Leocádio da Silva Júnior</t>
         </is>
       </c>
-      <c r="V130" t="inlineStr"/>
+      <c r="V130" t="n">
+        <v/>
+      </c>
       <c r="W130" t="inlineStr">
         <is>
           <t>Não foi possível enviar o arquivo por motivos do documento exceder 10MB</t>
@@ -19256,16 +19258,30 @@
       </c>
       <c r="Z130" t="inlineStr">
         <is>
-          <t>Integração nova</t>
-        </is>
-      </c>
-      <c r="AA130" t="inlineStr"/>
-      <c r="AB130" t="inlineStr"/>
-      <c r="AC130" t="inlineStr"/>
-      <c r="AD130" t="inlineStr"/>
-      <c r="AE130" t="inlineStr"/>
-      <c r="AF130" t="inlineStr"/>
-      <c r="AG130" t="inlineStr"/>
+          <t>Integração nova (16/06)</t>
+        </is>
+      </c>
+      <c r="AA130" t="n">
+        <v/>
+      </c>
+      <c r="AB130" t="n">
+        <v/>
+      </c>
+      <c r="AC130" t="n">
+        <v/>
+      </c>
+      <c r="AD130" t="n">
+        <v/>
+      </c>
+      <c r="AE130" t="n">
+        <v/>
+      </c>
+      <c r="AF130" t="n">
+        <v/>
+      </c>
+      <c r="AG130" t="n">
+        <v/>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -19298,7 +19314,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Prof. Maxim Repetto</t>
+          <t>Prof. Dr. Maxim Repetto</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -19321,10 +19337,8 @@
           <t>Não informado</t>
         </is>
       </c>
-      <c r="L131" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
+      <c r="L131" t="n">
+        <v>33</v>
       </c>
       <c r="M131" t="inlineStr">
         <is>
@@ -19393,16 +19407,30 @@
       </c>
       <c r="Z131" t="inlineStr">
         <is>
-          <t>Integração nova</t>
-        </is>
-      </c>
-      <c r="AA131" t="inlineStr"/>
-      <c r="AB131" t="inlineStr"/>
-      <c r="AC131" t="inlineStr"/>
-      <c r="AD131" t="inlineStr"/>
-      <c r="AE131" t="inlineStr"/>
-      <c r="AF131" t="inlineStr"/>
-      <c r="AG131" t="inlineStr"/>
+          <t>Integração nova (16/06)</t>
+        </is>
+      </c>
+      <c r="AA131" t="n">
+        <v/>
+      </c>
+      <c r="AB131" t="n">
+        <v/>
+      </c>
+      <c r="AC131" t="n">
+        <v/>
+      </c>
+      <c r="AD131" t="n">
+        <v/>
+      </c>
+      <c r="AE131" t="n">
+        <v/>
+      </c>
+      <c r="AF131" t="n">
+        <v/>
+      </c>
+      <c r="AG131" t="n">
+        <v/>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -19458,10 +19486,8 @@
           <t>1º semestre</t>
         </is>
       </c>
-      <c r="L132" t="inlineStr">
-        <is>
-          <t>104</t>
-        </is>
+      <c r="L132" t="n">
+        <v>104</v>
       </c>
       <c r="M132" t="inlineStr">
         <is>
@@ -19530,16 +19556,30 @@
       </c>
       <c r="Z132" t="inlineStr">
         <is>
-          <t>Integração nova</t>
-        </is>
-      </c>
-      <c r="AA132" t="inlineStr"/>
-      <c r="AB132" t="inlineStr"/>
-      <c r="AC132" t="inlineStr"/>
-      <c r="AD132" t="inlineStr"/>
-      <c r="AE132" t="inlineStr"/>
-      <c r="AF132" t="inlineStr"/>
-      <c r="AG132" t="inlineStr"/>
+          <t>Integração nova (16/06)</t>
+        </is>
+      </c>
+      <c r="AA132" t="n">
+        <v/>
+      </c>
+      <c r="AB132" t="n">
+        <v/>
+      </c>
+      <c r="AC132" t="n">
+        <v/>
+      </c>
+      <c r="AD132" t="n">
+        <v/>
+      </c>
+      <c r="AE132" t="n">
+        <v/>
+      </c>
+      <c r="AF132" t="n">
+        <v/>
+      </c>
+      <c r="AG132" t="n">
+        <v/>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -19595,10 +19635,8 @@
           <t>2º semestre</t>
         </is>
       </c>
-      <c r="L133" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
+      <c r="L133" t="n">
+        <v>34</v>
       </c>
       <c r="M133" t="inlineStr">
         <is>
@@ -19650,7 +19688,9 @@
           <t>Não se aplica</t>
         </is>
       </c>
-      <c r="W133" t="inlineStr"/>
+      <c r="W133" t="n">
+        <v/>
+      </c>
       <c r="X133" t="inlineStr">
         <is>
           <t>13/06/2026 17:14:10</t>
@@ -19663,16 +19703,30 @@
       </c>
       <c r="Z133" t="inlineStr">
         <is>
-          <t>Integração nova</t>
-        </is>
-      </c>
-      <c r="AA133" t="inlineStr"/>
-      <c r="AB133" t="inlineStr"/>
-      <c r="AC133" t="inlineStr"/>
-      <c r="AD133" t="inlineStr"/>
-      <c r="AE133" t="inlineStr"/>
-      <c r="AF133" t="inlineStr"/>
-      <c r="AG133" t="inlineStr"/>
+          <t>Integração nova (16/06)</t>
+        </is>
+      </c>
+      <c r="AA133" t="n">
+        <v/>
+      </c>
+      <c r="AB133" t="n">
+        <v/>
+      </c>
+      <c r="AC133" t="n">
+        <v/>
+      </c>
+      <c r="AD133" t="n">
+        <v/>
+      </c>
+      <c r="AE133" t="n">
+        <v/>
+      </c>
+      <c r="AF133" t="n">
+        <v/>
+      </c>
+      <c r="AG133" t="n">
+        <v/>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -19728,10 +19782,8 @@
           <t>Não informado</t>
         </is>
       </c>
-      <c r="L134" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
+      <c r="L134" t="n">
+        <v>44</v>
       </c>
       <c r="M134" t="inlineStr">
         <is>
@@ -19800,16 +19852,30 @@
       </c>
       <c r="Z134" t="inlineStr">
         <is>
-          <t>Integração nova</t>
-        </is>
-      </c>
-      <c r="AA134" t="inlineStr"/>
-      <c r="AB134" t="inlineStr"/>
-      <c r="AC134" t="inlineStr"/>
-      <c r="AD134" t="inlineStr"/>
-      <c r="AE134" t="inlineStr"/>
-      <c r="AF134" t="inlineStr"/>
-      <c r="AG134" t="inlineStr"/>
+          <t>Integração nova (16/06)</t>
+        </is>
+      </c>
+      <c r="AA134" t="n">
+        <v/>
+      </c>
+      <c r="AB134" t="n">
+        <v/>
+      </c>
+      <c r="AC134" t="n">
+        <v/>
+      </c>
+      <c r="AD134" t="n">
+        <v/>
+      </c>
+      <c r="AE134" t="n">
+        <v/>
+      </c>
+      <c r="AF134" t="n">
+        <v/>
+      </c>
+      <c r="AG134" t="n">
+        <v/>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -19865,10 +19931,8 @@
           <t>Não informado</t>
         </is>
       </c>
-      <c r="L135" t="inlineStr">
-        <is>
-          <t>38</t>
-        </is>
+      <c r="L135" t="n">
+        <v>38</v>
       </c>
       <c r="M135" t="inlineStr">
         <is>
@@ -19937,16 +20001,30 @@
       </c>
       <c r="Z135" t="inlineStr">
         <is>
-          <t>Integração nova</t>
-        </is>
-      </c>
-      <c r="AA135" t="inlineStr"/>
-      <c r="AB135" t="inlineStr"/>
-      <c r="AC135" t="inlineStr"/>
-      <c r="AD135" t="inlineStr"/>
-      <c r="AE135" t="inlineStr"/>
-      <c r="AF135" t="inlineStr"/>
-      <c r="AG135" t="inlineStr"/>
+          <t>Integração nova (16/06)</t>
+        </is>
+      </c>
+      <c r="AA135" t="n">
+        <v/>
+      </c>
+      <c r="AB135" t="n">
+        <v/>
+      </c>
+      <c r="AC135" t="n">
+        <v/>
+      </c>
+      <c r="AD135" t="n">
+        <v/>
+      </c>
+      <c r="AE135" t="n">
+        <v/>
+      </c>
+      <c r="AF135" t="n">
+        <v/>
+      </c>
+      <c r="AG135" t="n">
+        <v/>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -19979,7 +20057,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>Prof. Dr. Jonildo Viana dos Santos</t>
+          <t>Prof. Dr. Jonildo Viana dos Santos.</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
@@ -20002,10 +20080,8 @@
           <t>Não informado</t>
         </is>
       </c>
-      <c r="L136" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
+      <c r="L136" t="n">
+        <v>30</v>
       </c>
       <c r="M136" t="inlineStr">
         <is>
@@ -20074,16 +20150,30 @@
       </c>
       <c r="Z136" t="inlineStr">
         <is>
-          <t>Integração nova</t>
-        </is>
-      </c>
-      <c r="AA136" t="inlineStr"/>
-      <c r="AB136" t="inlineStr"/>
-      <c r="AC136" t="inlineStr"/>
-      <c r="AD136" t="inlineStr"/>
-      <c r="AE136" t="inlineStr"/>
-      <c r="AF136" t="inlineStr"/>
-      <c r="AG136" t="inlineStr"/>
+          <t>Integração nova (16/06)</t>
+        </is>
+      </c>
+      <c r="AA136" t="n">
+        <v/>
+      </c>
+      <c r="AB136" t="n">
+        <v/>
+      </c>
+      <c r="AC136" t="n">
+        <v/>
+      </c>
+      <c r="AD136" t="n">
+        <v/>
+      </c>
+      <c r="AE136" t="n">
+        <v/>
+      </c>
+      <c r="AF136" t="n">
+        <v/>
+      </c>
+      <c r="AG136" t="n">
+        <v/>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -20139,10 +20229,8 @@
           <t>Não informado</t>
         </is>
       </c>
-      <c r="L137" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
+      <c r="L137" t="n">
+        <v>33</v>
       </c>
       <c r="M137" t="inlineStr">
         <is>
@@ -20211,16 +20299,30 @@
       </c>
       <c r="Z137" t="inlineStr">
         <is>
-          <t>Integração nova</t>
-        </is>
-      </c>
-      <c r="AA137" t="inlineStr"/>
-      <c r="AB137" t="inlineStr"/>
-      <c r="AC137" t="inlineStr"/>
-      <c r="AD137" t="inlineStr"/>
-      <c r="AE137" t="inlineStr"/>
-      <c r="AF137" t="inlineStr"/>
-      <c r="AG137" t="inlineStr"/>
+          <t>Integração nova (16/06)</t>
+        </is>
+      </c>
+      <c r="AA137" t="n">
+        <v/>
+      </c>
+      <c r="AB137" t="n">
+        <v/>
+      </c>
+      <c r="AC137" t="n">
+        <v/>
+      </c>
+      <c r="AD137" t="n">
+        <v/>
+      </c>
+      <c r="AE137" t="n">
+        <v/>
+      </c>
+      <c r="AF137" t="n">
+        <v/>
+      </c>
+      <c r="AG137" t="n">
+        <v/>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -20276,10 +20378,8 @@
           <t>Não informado</t>
         </is>
       </c>
-      <c r="L138" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
+      <c r="L138" t="n">
+        <v>32</v>
       </c>
       <c r="M138" t="inlineStr">
         <is>
@@ -20348,16 +20448,30 @@
       </c>
       <c r="Z138" t="inlineStr">
         <is>
-          <t>Integração nova</t>
-        </is>
-      </c>
-      <c r="AA138" t="inlineStr"/>
-      <c r="AB138" t="inlineStr"/>
-      <c r="AC138" t="inlineStr"/>
-      <c r="AD138" t="inlineStr"/>
-      <c r="AE138" t="inlineStr"/>
-      <c r="AF138" t="inlineStr"/>
-      <c r="AG138" t="inlineStr"/>
+          <t>Integração nova (16/06)</t>
+        </is>
+      </c>
+      <c r="AA138" t="n">
+        <v/>
+      </c>
+      <c r="AB138" t="n">
+        <v/>
+      </c>
+      <c r="AC138" t="n">
+        <v/>
+      </c>
+      <c r="AD138" t="n">
+        <v/>
+      </c>
+      <c r="AE138" t="n">
+        <v/>
+      </c>
+      <c r="AF138" t="n">
+        <v/>
+      </c>
+      <c r="AG138" t="n">
+        <v/>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -20413,10 +20527,8 @@
           <t>Não informado</t>
         </is>
       </c>
-      <c r="L139" t="inlineStr">
-        <is>
-          <t>48</t>
-        </is>
+      <c r="L139" t="n">
+        <v>48</v>
       </c>
       <c r="M139" t="inlineStr">
         <is>
@@ -20485,16 +20597,30 @@
       </c>
       <c r="Z139" t="inlineStr">
         <is>
-          <t>Integração nova</t>
-        </is>
-      </c>
-      <c r="AA139" t="inlineStr"/>
-      <c r="AB139" t="inlineStr"/>
-      <c r="AC139" t="inlineStr"/>
-      <c r="AD139" t="inlineStr"/>
-      <c r="AE139" t="inlineStr"/>
-      <c r="AF139" t="inlineStr"/>
-      <c r="AG139" t="inlineStr"/>
+          <t>Integração nova (16/06)</t>
+        </is>
+      </c>
+      <c r="AA139" t="n">
+        <v/>
+      </c>
+      <c r="AB139" t="n">
+        <v/>
+      </c>
+      <c r="AC139" t="n">
+        <v/>
+      </c>
+      <c r="AD139" t="n">
+        <v/>
+      </c>
+      <c r="AE139" t="n">
+        <v/>
+      </c>
+      <c r="AF139" t="n">
+        <v/>
+      </c>
+      <c r="AG139" t="n">
+        <v/>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -20550,10 +20676,8 @@
           <t>Não informado</t>
         </is>
       </c>
-      <c r="L140" t="inlineStr">
-        <is>
-          <t>37</t>
-        </is>
+      <c r="L140" t="n">
+        <v>37</v>
       </c>
       <c r="M140" t="inlineStr">
         <is>
@@ -20600,7 +20724,9 @@
           <t>Elcio Leocádio da Silva Júnior</t>
         </is>
       </c>
-      <c r="V140" t="inlineStr"/>
+      <c r="V140" t="n">
+        <v/>
+      </c>
       <c r="W140" t="inlineStr">
         <is>
           <t>A pasta do drive diz ser de 2021 mas o TCC é de 2019, também há muitos equívocos em formatação do próprio trabalho.</t>
@@ -20618,16 +20744,30 @@
       </c>
       <c r="Z140" t="inlineStr">
         <is>
-          <t>Integração nova</t>
-        </is>
-      </c>
-      <c r="AA140" t="inlineStr"/>
-      <c r="AB140" t="inlineStr"/>
-      <c r="AC140" t="inlineStr"/>
-      <c r="AD140" t="inlineStr"/>
-      <c r="AE140" t="inlineStr"/>
-      <c r="AF140" t="inlineStr"/>
-      <c r="AG140" t="inlineStr"/>
+          <t>Integração nova (16/06)</t>
+        </is>
+      </c>
+      <c r="AA140" t="n">
+        <v/>
+      </c>
+      <c r="AB140" t="n">
+        <v/>
+      </c>
+      <c r="AC140" t="n">
+        <v/>
+      </c>
+      <c r="AD140" t="n">
+        <v/>
+      </c>
+      <c r="AE140" t="n">
+        <v/>
+      </c>
+      <c r="AF140" t="n">
+        <v/>
+      </c>
+      <c r="AG140" t="n">
+        <v/>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -20660,7 +20800,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>Profa. MSc. Jovina Mafra dos Santos.</t>
+          <t>professora Mestre Jovina Mafra dos Santos.</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
@@ -20683,10 +20823,8 @@
           <t>Não informado</t>
         </is>
       </c>
-      <c r="L141" t="inlineStr">
-        <is>
-          <t>56</t>
-        </is>
+      <c r="L141" t="n">
+        <v>56</v>
       </c>
       <c r="M141" t="inlineStr">
         <is>
@@ -20733,8 +20871,12 @@
           <t>Elcio Leocádio da Silva Júnior</t>
         </is>
       </c>
-      <c r="V141" t="inlineStr"/>
-      <c r="W141" t="inlineStr"/>
+      <c r="V141" t="n">
+        <v/>
+      </c>
+      <c r="W141" t="n">
+        <v/>
+      </c>
       <c r="X141" t="inlineStr">
         <is>
           <t>16/06/2026 19:21:49</t>
@@ -20747,16 +20889,30 @@
       </c>
       <c r="Z141" t="inlineStr">
         <is>
-          <t>Integração nova</t>
-        </is>
-      </c>
-      <c r="AA141" t="inlineStr"/>
-      <c r="AB141" t="inlineStr"/>
-      <c r="AC141" t="inlineStr"/>
-      <c r="AD141" t="inlineStr"/>
-      <c r="AE141" t="inlineStr"/>
-      <c r="AF141" t="inlineStr"/>
-      <c r="AG141" t="inlineStr"/>
+          <t>Integração nova (16/06)</t>
+        </is>
+      </c>
+      <c r="AA141" t="n">
+        <v/>
+      </c>
+      <c r="AB141" t="n">
+        <v/>
+      </c>
+      <c r="AC141" t="n">
+        <v/>
+      </c>
+      <c r="AD141" t="n">
+        <v/>
+      </c>
+      <c r="AE141" t="n">
+        <v/>
+      </c>
+      <c r="AF141" t="n">
+        <v/>
+      </c>
+      <c r="AG141" t="n">
+        <v/>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -20812,10 +20968,8 @@
           <t>2º semestre</t>
         </is>
       </c>
-      <c r="L142" t="inlineStr">
-        <is>
-          <t>38</t>
-        </is>
+      <c r="L142" t="n">
+        <v>38</v>
       </c>
       <c r="M142" t="inlineStr">
         <is>
@@ -20862,8 +21016,12 @@
           <t>Elcio Leocádio da Silva Júnior</t>
         </is>
       </c>
-      <c r="V142" t="inlineStr"/>
-      <c r="W142" t="inlineStr"/>
+      <c r="V142" t="n">
+        <v/>
+      </c>
+      <c r="W142" t="n">
+        <v/>
+      </c>
       <c r="X142" t="inlineStr">
         <is>
           <t>16/06/2026 19:31:19</t>
@@ -20876,16 +21034,30 @@
       </c>
       <c r="Z142" t="inlineStr">
         <is>
-          <t>Integração nova</t>
-        </is>
-      </c>
-      <c r="AA142" t="inlineStr"/>
-      <c r="AB142" t="inlineStr"/>
-      <c r="AC142" t="inlineStr"/>
-      <c r="AD142" t="inlineStr"/>
-      <c r="AE142" t="inlineStr"/>
-      <c r="AF142" t="inlineStr"/>
-      <c r="AG142" t="inlineStr"/>
+          <t>Integração nova (16/06)</t>
+        </is>
+      </c>
+      <c r="AA142" t="n">
+        <v/>
+      </c>
+      <c r="AB142" t="n">
+        <v/>
+      </c>
+      <c r="AC142" t="n">
+        <v/>
+      </c>
+      <c r="AD142" t="n">
+        <v/>
+      </c>
+      <c r="AE142" t="n">
+        <v/>
+      </c>
+      <c r="AF142" t="n">
+        <v/>
+      </c>
+      <c r="AG142" t="n">
+        <v/>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -20941,10 +21113,8 @@
           <t>1º semestre</t>
         </is>
       </c>
-      <c r="L143" t="inlineStr">
-        <is>
-          <t>64</t>
-        </is>
+      <c r="L143" t="n">
+        <v>64</v>
       </c>
       <c r="M143" t="inlineStr">
         <is>
@@ -20991,8 +21161,12 @@
           <t>Elcio Leocádio da Silva Júnior</t>
         </is>
       </c>
-      <c r="V143" t="inlineStr"/>
-      <c r="W143" t="inlineStr"/>
+      <c r="V143" t="n">
+        <v/>
+      </c>
+      <c r="W143" t="n">
+        <v/>
+      </c>
       <c r="X143" t="inlineStr">
         <is>
           <t>16/06/2026 19:39:46</t>
@@ -21005,16 +21179,30 @@
       </c>
       <c r="Z143" t="inlineStr">
         <is>
-          <t>Integração nova</t>
-        </is>
-      </c>
-      <c r="AA143" t="inlineStr"/>
-      <c r="AB143" t="inlineStr"/>
-      <c r="AC143" t="inlineStr"/>
-      <c r="AD143" t="inlineStr"/>
-      <c r="AE143" t="inlineStr"/>
-      <c r="AF143" t="inlineStr"/>
-      <c r="AG143" t="inlineStr"/>
+          <t>Integração nova (16/06)</t>
+        </is>
+      </c>
+      <c r="AA143" t="n">
+        <v/>
+      </c>
+      <c r="AB143" t="n">
+        <v/>
+      </c>
+      <c r="AC143" t="n">
+        <v/>
+      </c>
+      <c r="AD143" t="n">
+        <v/>
+      </c>
+      <c r="AE143" t="n">
+        <v/>
+      </c>
+      <c r="AF143" t="n">
+        <v/>
+      </c>
+      <c r="AG143" t="n">
+        <v/>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -21070,10 +21258,8 @@
           <t>2º semestre</t>
         </is>
       </c>
-      <c r="L144" t="inlineStr">
-        <is>
-          <t>64</t>
-        </is>
+      <c r="L144" t="n">
+        <v>64</v>
       </c>
       <c r="M144" t="inlineStr">
         <is>
@@ -21120,7 +21306,9 @@
           <t>Elcio Leocádio da Silva Júnior</t>
         </is>
       </c>
-      <c r="V144" t="inlineStr"/>
+      <c r="V144" t="n">
+        <v/>
+      </c>
       <c r="W144" t="inlineStr">
         <is>
           <t>A data da capa diz 2022, mas a aprovação (que consta no documento) diz 16 de novembro de 2021</t>
@@ -21138,16 +21326,30 @@
       </c>
       <c r="Z144" t="inlineStr">
         <is>
-          <t>Integração nova</t>
-        </is>
-      </c>
-      <c r="AA144" t="inlineStr"/>
-      <c r="AB144" t="inlineStr"/>
-      <c r="AC144" t="inlineStr"/>
-      <c r="AD144" t="inlineStr"/>
-      <c r="AE144" t="inlineStr"/>
-      <c r="AF144" t="inlineStr"/>
-      <c r="AG144" t="inlineStr"/>
+          <t>Integração nova (16/06)</t>
+        </is>
+      </c>
+      <c r="AA144" t="n">
+        <v/>
+      </c>
+      <c r="AB144" t="n">
+        <v/>
+      </c>
+      <c r="AC144" t="n">
+        <v/>
+      </c>
+      <c r="AD144" t="n">
+        <v/>
+      </c>
+      <c r="AE144" t="n">
+        <v/>
+      </c>
+      <c r="AF144" t="n">
+        <v/>
+      </c>
+      <c r="AG144" t="n">
+        <v/>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -21203,10 +21405,8 @@
           <t>Não informado</t>
         </is>
       </c>
-      <c r="L145" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
+      <c r="L145" t="n">
+        <v>34</v>
       </c>
       <c r="M145" t="inlineStr">
         <is>
@@ -21253,8 +21453,12 @@
           <t>Elcio Leocádio da Silva Júnior</t>
         </is>
       </c>
-      <c r="V145" t="inlineStr"/>
-      <c r="W145" t="inlineStr"/>
+      <c r="V145" t="n">
+        <v/>
+      </c>
+      <c r="W145" t="n">
+        <v/>
+      </c>
       <c r="X145" t="inlineStr">
         <is>
           <t>16/06/2026 19:59:32</t>
@@ -21267,16 +21471,30 @@
       </c>
       <c r="Z145" t="inlineStr">
         <is>
-          <t>Integração nova</t>
-        </is>
-      </c>
-      <c r="AA145" t="inlineStr"/>
-      <c r="AB145" t="inlineStr"/>
-      <c r="AC145" t="inlineStr"/>
-      <c r="AD145" t="inlineStr"/>
-      <c r="AE145" t="inlineStr"/>
-      <c r="AF145" t="inlineStr"/>
-      <c r="AG145" t="inlineStr"/>
+          <t>Integração nova (16/06)</t>
+        </is>
+      </c>
+      <c r="AA145" t="n">
+        <v/>
+      </c>
+      <c r="AB145" t="n">
+        <v/>
+      </c>
+      <c r="AC145" t="n">
+        <v/>
+      </c>
+      <c r="AD145" t="n">
+        <v/>
+      </c>
+      <c r="AE145" t="n">
+        <v/>
+      </c>
+      <c r="AF145" t="n">
+        <v/>
+      </c>
+      <c r="AG145" t="n">
+        <v/>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -21332,10 +21550,8 @@
           <t>1º semestre</t>
         </is>
       </c>
-      <c r="L146" t="inlineStr">
-        <is>
-          <t>48</t>
-        </is>
+      <c r="L146" t="n">
+        <v>48</v>
       </c>
       <c r="M146" t="inlineStr">
         <is>
@@ -21404,16 +21620,30 @@
       </c>
       <c r="Z146" t="inlineStr">
         <is>
-          <t>Integração nova</t>
-        </is>
-      </c>
-      <c r="AA146" t="inlineStr"/>
-      <c r="AB146" t="inlineStr"/>
-      <c r="AC146" t="inlineStr"/>
-      <c r="AD146" t="inlineStr"/>
-      <c r="AE146" t="inlineStr"/>
-      <c r="AF146" t="inlineStr"/>
-      <c r="AG146" t="inlineStr"/>
+          <t>Integração nova (16/06)</t>
+        </is>
+      </c>
+      <c r="AA146" t="n">
+        <v/>
+      </c>
+      <c r="AB146" t="n">
+        <v/>
+      </c>
+      <c r="AC146" t="n">
+        <v/>
+      </c>
+      <c r="AD146" t="n">
+        <v/>
+      </c>
+      <c r="AE146" t="n">
+        <v/>
+      </c>
+      <c r="AF146" t="n">
+        <v/>
+      </c>
+      <c r="AG146" t="n">
+        <v/>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -21469,10 +21699,8 @@
           <t>2º semestre</t>
         </is>
       </c>
-      <c r="L147" t="inlineStr">
-        <is>
-          <t>51</t>
-        </is>
+      <c r="L147" t="n">
+        <v>51</v>
       </c>
       <c r="M147" t="inlineStr">
         <is>
@@ -21524,7 +21752,9 @@
           <t>não se aplica</t>
         </is>
       </c>
-      <c r="W147" t="inlineStr"/>
+      <c r="W147" t="n">
+        <v/>
+      </c>
       <c r="X147" t="inlineStr">
         <is>
           <t>16/06/2026 22:59:28</t>
@@ -21537,16 +21767,30 @@
       </c>
       <c r="Z147" t="inlineStr">
         <is>
-          <t>Integração nova</t>
-        </is>
-      </c>
-      <c r="AA147" t="inlineStr"/>
-      <c r="AB147" t="inlineStr"/>
-      <c r="AC147" t="inlineStr"/>
-      <c r="AD147" t="inlineStr"/>
-      <c r="AE147" t="inlineStr"/>
-      <c r="AF147" t="inlineStr"/>
-      <c r="AG147" t="inlineStr"/>
+          <t>Integração nova (16/06)</t>
+        </is>
+      </c>
+      <c r="AA147" t="n">
+        <v/>
+      </c>
+      <c r="AB147" t="n">
+        <v/>
+      </c>
+      <c r="AC147" t="n">
+        <v/>
+      </c>
+      <c r="AD147" t="n">
+        <v/>
+      </c>
+      <c r="AE147" t="n">
+        <v/>
+      </c>
+      <c r="AF147" t="n">
+        <v/>
+      </c>
+      <c r="AG147" t="n">
+        <v/>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -21579,7 +21823,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>Prof. Dr. Jaci Guilherme Vieira</t>
+          <t>Prof. Dr. Jaci Guilherme  Vieira.</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
@@ -21602,10 +21846,8 @@
           <t>1º semestre</t>
         </is>
       </c>
-      <c r="L148" t="inlineStr">
-        <is>
-          <t>105</t>
-        </is>
+      <c r="L148" t="n">
+        <v>105</v>
       </c>
       <c r="M148" t="inlineStr">
         <is>
@@ -21657,7 +21899,9 @@
           <t>Não se aplica</t>
         </is>
       </c>
-      <c r="W148" t="inlineStr"/>
+      <c r="W148" t="n">
+        <v/>
+      </c>
       <c r="X148" t="inlineStr">
         <is>
           <t>16/06/2026 23:17:11</t>
@@ -21670,16 +21914,30 @@
       </c>
       <c r="Z148" t="inlineStr">
         <is>
-          <t>Integração nova</t>
-        </is>
-      </c>
-      <c r="AA148" t="inlineStr"/>
-      <c r="AB148" t="inlineStr"/>
-      <c r="AC148" t="inlineStr"/>
-      <c r="AD148" t="inlineStr"/>
-      <c r="AE148" t="inlineStr"/>
-      <c r="AF148" t="inlineStr"/>
-      <c r="AG148" t="inlineStr"/>
+          <t>Integração nova (16/06)</t>
+        </is>
+      </c>
+      <c r="AA148" t="n">
+        <v/>
+      </c>
+      <c r="AB148" t="n">
+        <v/>
+      </c>
+      <c r="AC148" t="n">
+        <v/>
+      </c>
+      <c r="AD148" t="n">
+        <v/>
+      </c>
+      <c r="AE148" t="n">
+        <v/>
+      </c>
+      <c r="AF148" t="n">
+        <v/>
+      </c>
+      <c r="AG148" t="n">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Limpar nomes de orientadores: 111 → 71 únicos (remover títulos e consolidar)
</commit_message>
<xml_diff>
--- a/outputs/analise/corpus_tccs_analisado.xlsx
+++ b/outputs/analise/corpus_tccs_analisado.xlsx
@@ -51,9 +51,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -421,41 +419,6 @@
   </sheetPr>
   <dimension ref="A1:AG148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="80" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
-    <col width="16" customWidth="1" min="22" max="22"/>
-    <col width="16" customWidth="1" min="23" max="23"/>
-    <col width="16" customWidth="1" min="24" max="24"/>
-    <col width="16" customWidth="1" min="25" max="25"/>
-    <col width="16" customWidth="1" min="26" max="26"/>
-    <col width="40" customWidth="1" min="27" max="27"/>
-    <col width="16" customWidth="1" min="28" max="28"/>
-    <col width="16" customWidth="1" min="29" max="29"/>
-    <col width="16" customWidth="1" min="30" max="30"/>
-    <col width="16" customWidth="1" min="31" max="31"/>
-    <col width="16" customWidth="1" min="32" max="32"/>
-    <col width="16" customWidth="1" min="33" max="33"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -655,7 +618,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor José García Mendoza</t>
+          <t>Dr. Héctor José García Mendoza</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -804,7 +767,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor José García Mendoza</t>
+          <t>Dr. Héctor José García Mendoza</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -953,7 +916,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor José García  Mendoza</t>
+          <t>Dr. Héctor José García Mendoza</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1102,7 +1065,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor José García Mendoza</t>
+          <t>Dr. Héctor José García Mendoza</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1251,7 +1214,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>bancaProfa Me. Mariana Souza da Cunha  Licenciatura Intercultural/Orientadora/UFRR</t>
+          <t>Mariana Souza da Cunha</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1396,7 +1359,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Dr. Ricardo Carvalho dos Santos.</t>
+          <t>Dr. Ricardo Carvalho dos Santos</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1541,7 +1504,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Dr. Ricardo Carvalho dos Santos.</t>
+          <t>Dr. Ricardo Carvalho dos Santos</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1686,7 +1649,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Dr. Ricardo Carvalho dos Santos.</t>
+          <t>Dr. Ricardo Carvalho dos Santos</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1831,7 +1794,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Orientadora Ananda Machado</t>
+          <t>Ananda Machado</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1976,7 +1939,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Dr. Ricardo Carvalho dos Santos.</t>
+          <t>Dr. Ricardo Carvalho dos Santos</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -2266,7 +2229,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>prof. Dr. Eliabe Procópio</t>
+          <t>Dr. Eliabe Procópio</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -2411,7 +2374,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Prof.a Dr.a Eliaine de Morais Belford Gomes</t>
+          <t>Eliaine de Morais Belford Gomes</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -2558,7 +2521,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Profa. Dra. Martha Julia Martins de Souza Orientadora/Curso de Letras - CCL/UFRR</t>
+          <t>Martha Julia Martins de Souza</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2703,7 +2666,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Prof.a Dr.a Sandra Moraes da Silva Cardozo.</t>
+          <t>Sandra Moraes da Silva Cardozo</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2848,7 +2811,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Prof.a Dr.a Eliaine de Morais Belford Gomes</t>
+          <t>Eliaine de Morais Belford Gomes</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2993,7 +2956,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Prof.a Dr.a Eliaine de Morais Belford Gomes</t>
+          <t>Eliaine de Morais Belford Gomes</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -3138,7 +3101,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor José García Mendoza</t>
+          <t>Dr. Héctor José García Mendoza</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -3287,7 +3250,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Prof. Dr. Sérgio Luiz Lopes</t>
+          <t>Dr. Sérgio Luiz Lopes</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -3432,7 +3395,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Prof.ª Dra. Cinara Franco Rechico Barberena</t>
+          <t>Cinara Franco Rechico Barberena</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -3577,7 +3540,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Prof. Dr. Flávio Corsini Lirio</t>
+          <t>Dr. Flávio Corsini Lirio</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -3724,7 +3687,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Alessandra Peternella Doutora em Educação, Universidade Federal de Roraima, Brasil.</t>
+          <t>Alessandra Peternella Doutora em Educação, Universidade Federal de Roraima, Brasil</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -3873,7 +3836,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Prof.o Dr. João Paulino da Silva Neto.</t>
+          <t>Dr. João Paulino da Silva Neto</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -4020,7 +3983,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Prof Dr. Maxim Repetto.</t>
+          <t>Dr. Maxim Repetto</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -4169,7 +4132,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Dra. Iana dos Santos Vasconcelos</t>
+          <t>Iana dos Santos Vasconcelos</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -4318,7 +4281,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Dra. Iana dos Santos Vasconcelos</t>
+          <t>Iana dos Santos Vasconcelos</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -4465,7 +4428,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Prof Dr. Maxim Repetto.</t>
+          <t>Dr. Maxim Repetto</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -4614,7 +4577,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Prof. Dr. Maxim Repetto Carrreno</t>
+          <t>Maxim Repetto Carreno</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -5206,7 +5169,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Profº Msc. Dr. Sebastião Oliveira Monteiro</t>
+          <t>Dr. Sebastião Monteiro Oliveira2</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -5643,7 +5606,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Profª Dr. Edlauva Oliveira dos Santos</t>
+          <t>Edlauva Oliveira dos Santos</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -5788,7 +5751,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Prof.a Dr.a Edlauva Oliveira dos Santos</t>
+          <t>Edlauva Oliveira dos Santos</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -6078,7 +6041,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Prof.o Dr. João Paulino da Silva Neto.</t>
+          <t>João Paulino da Silva Neto</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -6368,7 +6331,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Prof.o Dr. João Paulino da Silva Neto.</t>
+          <t>Dr. João Paulino da Silva Neto</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -6513,7 +6476,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Prof.o Dr. João Paulino da Silva Neto.</t>
+          <t>Dr. João Paulino da Silva Neto</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -6658,7 +6621,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Maria Edith Romano Siems Professora do Centro de Educação da Universidade Federal de Roraima e Pedagoga pela Faculdade de Filosofia Ciências e Letras de Sorocaba, com mestrado em Educação pela Universidade Federal de Juiz de Fora, com doutorado em Educação Especial (Educação do Indivíduo Especial) pela Universidade Federal de São Carlos e pós-doutorado em Educação pelo Instituto de Educação da Universidade de Lisboa.</t>
+          <t>Maria Edith Romano Siems Professora do Centro de Educação da Universidade Federal de Roraima e Pedagoga pela Faculdade de Filosofia Ciências e Letras de Sorocaba, com mestrado em Educação pela Universidade Federal de Juiz de Fora, com doutorado em Educação Especial (Educação do Indivíduo Especial) pela Universidade Federal de São Carlos e pós-doutorado em Educação pelo Instituto de Educação da Universidade de Lisboa</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -6803,7 +6766,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Prof. Dra. Gilvete de Lima Gabriel</t>
+          <t>Dra. Gilvete de Lima Gabriel</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -6948,7 +6911,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Prof. Dr. Pedro Augusto Hercks Menin</t>
+          <t>Pedro Augusto Hercks Menin</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -7236,7 +7199,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Prof. Dr. Sebastião Monteiro Oliveira</t>
+          <t>Dr. Sebastião Monteiro Oliveira</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -7381,7 +7344,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Prof.a Dr.a Edlauva Oliveira dos Santos</t>
+          <t>Edlauva Oliveira dos Santos</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -7816,7 +7779,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Profª Ma. Danielle Trindade</t>
+          <t>Danielle Trindade</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -7961,7 +7924,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Profa. Dra. Zoraide  dos Anjos Gonçalves da Silva Vieira</t>
+          <t>Zoraide dos Anjos Gonçalves da Silva Vieira</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -8106,7 +8069,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Prof. Msc. Celino Alexandre Raposo</t>
+          <t>Me. Celino Alexandre Raposo</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -8251,7 +8214,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Prof.Dr. Fábio Almeida  de Carvalho</t>
+          <t>Dr. Fábio Almeida de Carvalho</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -8396,7 +8359,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Profa. Dra. Zoraide dos Anjos Gonçalves da Silva Vieira.</t>
+          <t>Zoraide dos Anjos Gonçalves Silva Vieira</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -8539,7 +8502,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Professora Ma. Naira Gomes Lamarão</t>
+          <t>Naira Gomes Lamarão</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -8682,7 +8645,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Prof. Msc. Celino Alexandre Raposo</t>
+          <t>Msc. Celino Alexandre Raposo</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -8825,7 +8788,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Profa Dra Ananda Machado.</t>
+          <t>Ananda Machado</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -8970,7 +8933,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Prof. Msc. Celino Alexandre Raposo</t>
+          <t>Msc. Celino Alexandre Raposo</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -9256,7 +9219,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Profa. Dra. Aurea Lúcia Melo Oliveira Corrêa.</t>
+          <t>Aurea Lúcia Melo Oliveira Corrêa</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -9687,7 +9650,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Prof.Dr. Fábio Almeida  de Carvalho</t>
+          <t>Fábio Almeida de Carvalho</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -9832,7 +9795,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Profa Dra Ananda Machado.</t>
+          <t>Ananda Machado</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -9977,7 +9940,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Professora Mestre Isabel Maria Fonseca</t>
+          <t>Isabel Maria Fonseca</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -10122,7 +10085,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Prof. Dr. Jonildo Viana dos Santos</t>
+          <t>Dr. Jonildo Viana dos Santos</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -10265,7 +10228,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Prof. Dr. Maxim Repetto</t>
+          <t>Dr. Maxim Repetto</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -10408,7 +10371,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Prof. Maxim Repetto</t>
+          <t>Dr. Maxim Repetto</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -10551,7 +10514,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Prof. Dr. Maxim Repetto</t>
+          <t>Dr. Maxim Repetto</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -10837,7 +10800,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Prof. Dr. Maxim Repetto Carrreno</t>
+          <t>Dr. Maxim Repetto Carrreno</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -10980,7 +10943,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Prof. Dr. Jonildo Viana  dos Santos.</t>
+          <t>Dr. Jonildo Viana dos Santos</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -11123,7 +11086,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Prof. Dr. Michael Lopes da Silva Rolim</t>
+          <t>Dr. Michael Lopes da Silva Rolim</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -11266,7 +11229,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Prof.a Me. Mariana Souza da Cunha.</t>
+          <t>Mariana Souza da Cunha</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -11409,7 +11372,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Prof.Dr. Fábio Almeida  de Carvalho</t>
+          <t>Fabíola Christian Almeida de Carvalho</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -11695,7 +11658,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Prof.ª Msc. Mariana Souza da Cunha</t>
+          <t>Me. Mariana Souza da Cunha</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -11838,7 +11801,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Dr. Ricardo Carvalho dos Santos.</t>
+          <t>Dr. Ricardo Carvalho dos Santos</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -11981,7 +11944,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Prof.a Mariana Souza da Cunha</t>
+          <t>Mariana Souza da Cunha</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -12124,7 +12087,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Prof.a Mariana Souza da Cunha</t>
+          <t>Mariana Souza da Cunha</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -12410,7 +12373,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Prof. Dr. Rafael Branquinho Abdala Norberto</t>
+          <t>Dr. Rafael Branquinho Abdala Norberto</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -12553,7 +12516,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Orientador: Prof. Dr. Jefferson Tiago de Souza Mendes da Silva</t>
+          <t>M.e Jefferson Tiago de Souza Mendes da Silva</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -12696,7 +12659,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Prof. Dr. Gustavo Frosi Benetti</t>
+          <t>Dr. Gustavo Frosi Benetti</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -12839,7 +12802,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Prof. Dra. Jéssica de Almeida</t>
+          <t>Jéssica de Almeida</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -12982,7 +12945,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Dr. José Rodrigo Santos Velho</t>
+          <t>José Rodrigo Santos Velho</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -13125,7 +13088,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Prof.a Dra Jéssica de Almeida</t>
+          <t>Jéssica de Almeida</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -13268,7 +13231,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Prof. Dr. Maxim Repetto</t>
+          <t>Dr. Maxim Repetto</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -13411,7 +13374,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Prof. M.E. Rafael Ricardo Friesen</t>
+          <t>M.E. Rafael Ricardo Friesen</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -13554,7 +13517,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Prof. Dr. Rafael Branquinho Abdala Norberto</t>
+          <t>Dr. Rafael Branquinho Abdala Norberto</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -13697,7 +13660,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Prof.a Dra Jéssica de Almeida</t>
+          <t>Dra. Jéssica de Almeida</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -13840,7 +13803,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Prof. Dra. Jéssica de Almeida</t>
+          <t>M.a. Jéssica de Almeida</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -13983,7 +13946,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Profa. Dra. Jéssica de Almeida.</t>
+          <t>Dra. Jessica de Almeida</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -14269,7 +14232,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Orientador: Prof. Dr. Jefferson Tiago de Souza Mendes da Silva</t>
+          <t>Jefferson Tiago de Souza Mendes da Silva</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -14412,7 +14375,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Prof. Dr. Rafael Branquinho Abdala Norberto</t>
+          <t>Dr. Rafael Branquinho Abdala Norberto</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -14555,7 +14518,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Prof. M.e Jefferson Tiago de Souza Mendes da Silva</t>
+          <t>Jefferson Tiago de Souza Mendes da Silva</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -14698,7 +14661,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Prof. Dr. Luciano Camargo</t>
+          <t>Dr. Luciano Camargo</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -14841,7 +14804,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Prof. Dr. Rafael Branquinho Abdala Norberto</t>
+          <t>Dr. Rafael Branquinho Abdala Norberto</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -14984,7 +14947,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Prof. Dr. Michael Lopes da Silva Rolim</t>
+          <t>Dr. Michael Lopes da Silva Rolim</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -15848,7 +15811,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Jovina Mafra dos Santos.</t>
+          <t>Jovina Mafra dos Santos</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -15991,7 +15954,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Profª. Mariana Cunha</t>
+          <t>Mariana Cunha</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
@@ -16134,7 +16097,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>Prof. Me. Rafael Friesen</t>
+          <t>Me. Rafael Friesen</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
@@ -16279,7 +16242,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>Prof. Dr. Rafael Branquinho Abdala Norberto</t>
+          <t>Dr. Rafael Branquinho Abdala Norberto</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -16424,7 +16387,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>Prof. Dr. Pedro Augusto Hercks Menin</t>
+          <t>Dr. Pedro Augusto Hercks Menin</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
@@ -16567,7 +16530,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>Prof. Dr. Sebastião Monteiro Oliveira</t>
+          <t>Sebastião Oliveira Monteiro</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
@@ -16710,7 +16673,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Prof.ª Dr.ª Maria Edith Romano Siems-Marcondes</t>
+          <t>Maria Edith Romano Siems Marcondes</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -16853,7 +16816,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Prof.ª Dra. Cinara Franco Rechico Barberena</t>
+          <t>Cinara Franco Rechico Barberena</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
@@ -16996,7 +16959,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Prof.ª Dr.ª Maria Edith Romano Siems-Marcondes</t>
+          <t>Maria Edith Romano Siems-Marcondes</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -17139,7 +17102,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Profa. M.ª MarianaSouzadaCunha</t>
+          <t>Mariana Souza da Cunha</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -17282,7 +17245,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>Professora Doutora Ise de Goreth Silva</t>
+          <t>Ise de Goreth Silva</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -17572,7 +17535,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>Prof. Dr. Michael Lopes da Silva Rolim</t>
+          <t>Michael Lopes da Silva Rolim</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -17717,7 +17680,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor José García Mendoza.</t>
+          <t>Dr. Héctor José García Mendoza</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -17862,7 +17825,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>Prof. Dr.  Héctor José García Mendoza.</t>
+          <t>Dr. Héctor José García Mendoza</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -18007,7 +17970,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor José García Mendoza</t>
+          <t>Dr. Héctor José García Mendoza</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -18152,7 +18115,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor  José García Mendoza</t>
+          <t>Dr. Héctor José García Mendoza</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -18297,7 +18260,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor  José García Mendoza</t>
+          <t>Dr. Héctor José García Mendoza</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -18442,7 +18405,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor  José García Mendoza</t>
+          <t>Dr. Héctor José García Mendoza</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -18587,7 +18550,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor José García Mendoza</t>
+          <t>Dr. Héctor José García Mendoza</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -18732,7 +18695,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor  José García Mendoza</t>
+          <t>Dr. Héctor José García Mendoza</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -18877,7 +18840,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>Prof. Dr. Héctor José García Mendoza</t>
+          <t>Dr. Héctor José García Mendoza</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -19022,7 +18985,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Prof. Dr.  Héctor José García Mendoza.</t>
+          <t>Dr. Héctor José García Mendoza</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -19169,7 +19132,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Profa. Dr. Moema  de Souza Esmeraldo</t>
+          <t>Moema de Souza Esmeraldo</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -19314,7 +19277,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Prof. Dr. Maxim Repetto</t>
+          <t>Maxim Repetto</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -19463,7 +19426,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>professor Doutor Maxim Repetto.</t>
+          <t>Maxim Repetto</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -19612,7 +19575,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>Profa. Dra. Zoraide  dos Anjos Gonçalves da Silva Vieira</t>
+          <t>Zoraide dos Anjos Gonçalves da Silva Vieira</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
@@ -19759,7 +19722,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>Prof. Dr. Fernando José Ciello</t>
+          <t>Dr. Fernando José Ciello</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -19908,7 +19871,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>Prof. Dr. Fernando José Ciello</t>
+          <t>Dr. Fernando José Ciello</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
@@ -20057,7 +20020,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>Prof. Dr. Jonildo Viana dos Santos.</t>
+          <t>Dr. Jonildo Viana dos Santos</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
@@ -20355,7 +20318,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>Prof. Dr. Jonildo Viana  dos Santos.</t>
+          <t>Dr. Jonildo Viana dos Santos</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -20504,7 +20467,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>Prof. Dr. Maxim Repetto</t>
+          <t>Dr. Maxim Repetto</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
@@ -20653,7 +20616,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>Prof. Dr. Michael Lopes da Silva Rolim</t>
+          <t>Dr. Michael Lopes da Silva Rolim</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
@@ -20800,7 +20763,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>professora Mestre Jovina Mafra dos Santos.</t>
+          <t>Jovina Mafra dos Santos</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
@@ -20945,7 +20908,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>Orientadora: Mariana Cunha</t>
+          <t>Mariana Cunha</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
@@ -21090,7 +21053,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>professora Mestre Jovina Mafra dos Santos.</t>
+          <t>Jovina Mafra dos Santos</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
@@ -21235,7 +21198,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>Orientadora: Profa. Mcs. Jovina Mafra dos Santos</t>
+          <t>Jovina Mafra dos Santos</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
@@ -21382,7 +21345,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>Orientadora: Profa Dra. Fabíola Christian Almeida de Carvalho</t>
+          <t>Fabíola Christian Almeida de Carvalho</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
@@ -21527,7 +21490,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>Prof. Dr. Jaci Guilherme  Vieira.</t>
+          <t>Dr. Jaci Guilherme Vieira</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
@@ -21676,7 +21639,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>Prof.a Dr.ª Francilene dos Santos Rodrigues.</t>
+          <t>Francilene dos Santos Rodrigues</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
@@ -21823,7 +21786,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>Prof. Dr. Jaci Guilherme  Vieira.</t>
+          <t>Dr. Jaci Guilherme Vieira</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">

</xml_diff>